<commit_message>
Three places where the repository disagreed with the dissertation
- vggt.yaml sat on image_mode: pad. Every reported VGGT run used crop,
  the upstream default; pad was the exp_171/172 ablation and was worse.
  The config had been left on the ablation's setting, so anyone
  reproducing from it got the variant the thesis rejected.
- The voxel IoU verdict still read "does not belong in chapter 5 ...
  leave it out of the results". It ended up as 5.8. The numbers were
  never in question - what the verdict measures is whether IoU reorders
  the methods, so say that, and name the criterion for what it tests.
- methodology_notes still described scale as a similarity fit against the
  LiDAR reference. That was true at exp_034 and is not what the final
  runs did: the 9.5 cm square fixes the unit, the object's own length
  follows from it, and registration is rigid.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tables/FINAL_results.xlsx
+++ b/docs/tables/FINAL_results.xlsx
@@ -3461,7 +3461,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Does not belong in chapter 5: IoU matches the F1@3cm ordering exactly on 2 of 6 objects, and every reordering it produces on the other 4 fails on inspection - see below. No new conclusion. Mention it in the methodology as an alternative that was considered, and leave it out of the results. The voxel sweep does reorder methods beyond the grid noise on bench_004, but singles out the same method ΔF1@10-3 already singles out there, so it restates the existing table rather than adding to it. Reorderings that were found but are smaller than the grid-origin noise, and so decide nothing: bench_004, bollard_003, bus_stop_002, information_sign_002. Caveat to state either way: the method ordering does not survive the grid-origin shift on bus_stop_002, information_sign_002, bench_004, bollard_003, so IoU cannot separate those methods at this voxel size.</t>
+          <t>IoU adds no ordering of its own: it matches the F1@3cm ordering exactly on 2 of 6 objects, and every reordering it produces on the other 4 fails on inspection - see below. So IoU confirms the F1 ordering rather than competing with it: a density-free check on the primary measure, not a second source of conclusions. The voxel sweep does reorder methods beyond the grid noise on bench_004, but singles out the same method ΔF1@10-3 already singles out there, so it restates the existing table rather than adding to it. Reorderings that were found but are smaller than the grid-origin noise, and so decide nothing: bench_004, bollard_003, bus_stop_002, information_sign_002. Caveat to state either way: the method ordering does not survive the grid-origin shift on bus_stop_002, information_sign_002, bench_004, bollard_003, so IoU cannot separate those methods at this voxel size.</t>
         </is>
       </c>
     </row>
@@ -8075,7 +8075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X16"/>
+  <dimension ref="A1:Y16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8097,11 +8097,12 @@
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="26" customWidth="1" min="18" max="18"/>
     <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="24" customWidth="1" min="22" max="22"/>
-    <col width="17" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="24" customWidth="1" min="23" max="23"/>
+    <col width="17" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8217,25 +8218,30 @@
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
+          <t>images in</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
           <t>reg-rate (%)</t>
         </is>
       </c>
-      <c r="U4" s="3" t="inlineStr">
+      <c r="V4" s="3" t="inlineStr">
         <is>
           <t>points raw</t>
         </is>
       </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="W4" s="3" t="inlineStr">
         <is>
           <t>points density-matched</t>
         </is>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="X4" s="3" t="inlineStr">
         <is>
           <t>excluded as gap</t>
         </is>
       </c>
-      <c r="X4" s="3" t="inlineStr">
+      <c r="Y4" s="3" t="inlineStr">
         <is>
           <t>DBSCAN (ft/eps/mp)</t>
         </is>
@@ -8308,18 +8314,21 @@
         <v>1.3</v>
       </c>
       <c r="T5" t="n">
+        <v>44</v>
+      </c>
+      <c r="U5" t="n">
         <v>100</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>105933</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>3847</v>
       </c>
-      <c r="W5" t="n">
+      <c r="X5" t="n">
         <v>754</v>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -8392,18 +8401,21 @@
         <v>1.11</v>
       </c>
       <c r="T6" t="n">
+        <v>44</v>
+      </c>
+      <c r="U6" t="n">
         <v>100</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>36609</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>2715</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>419</v>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -8476,18 +8488,21 @@
         <v>1.42</v>
       </c>
       <c r="T7" t="n">
+        <v>44</v>
+      </c>
+      <c r="U7" t="n">
         <v>100</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>167287</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>5592</v>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>1295</v>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -8560,18 +8575,21 @@
         <v>1.27</v>
       </c>
       <c r="T8" t="n">
+        <v>44</v>
+      </c>
+      <c r="U8" t="n">
         <v>100</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>441241</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>16196</v>
       </c>
-      <c r="W8" t="n">
+      <c r="X8" t="n">
         <v>4072</v>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -8644,18 +8662,21 @@
         <v>1.21</v>
       </c>
       <c r="T9" t="n">
+        <v>44</v>
+      </c>
+      <c r="U9" t="n">
         <v>100</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>750396</v>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>12872</v>
       </c>
-      <c r="W9" t="n">
+      <c r="X9" t="n">
         <v>2676</v>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -8728,18 +8749,21 @@
         <v>1.38</v>
       </c>
       <c r="T10" t="n">
+        <v>44</v>
+      </c>
+      <c r="U10" t="n">
         <v>100</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>482225</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>13029</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>2580</v>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -8812,18 +8836,21 @@
         <v>1.74</v>
       </c>
       <c r="T11" t="n">
+        <v>48</v>
+      </c>
+      <c r="U11" t="n">
         <v>100</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>547654</v>
       </c>
-      <c r="V11" t="n">
+      <c r="W11" t="n">
         <v>25404</v>
       </c>
-      <c r="W11" t="n">
+      <c r="X11" t="n">
         <v>14198</v>
       </c>
-      <c r="X11" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -8896,18 +8923,21 @@
         <v>1.95</v>
       </c>
       <c r="T12" t="n">
+        <v>48</v>
+      </c>
+      <c r="U12" t="n">
         <v>95.8</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
         <v>801528</v>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>19421</v>
       </c>
-      <c r="W12" t="n">
+      <c r="X12" t="n">
         <v>15582</v>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="Y12" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -8980,18 +9010,21 @@
         <v>1.96</v>
       </c>
       <c r="T13" t="n">
+        <v>48</v>
+      </c>
+      <c r="U13" t="n">
         <v>100</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
         <v>716317</v>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>35676</v>
       </c>
-      <c r="W13" t="n">
+      <c r="X13" t="n">
         <v>21922</v>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -9064,18 +9097,21 @@
         <v>1.73</v>
       </c>
       <c r="T14" t="n">
+        <v>48</v>
+      </c>
+      <c r="U14" t="n">
         <v>100</v>
       </c>
-      <c r="U14" t="n">
+      <c r="V14" t="n">
         <v>540530</v>
       </c>
-      <c r="V14" t="n">
+      <c r="W14" t="n">
         <v>75146</v>
       </c>
-      <c r="W14" t="n">
+      <c r="X14" t="n">
         <v>36753</v>
       </c>
-      <c r="X14" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -9148,18 +9184,21 @@
         <v>1.91</v>
       </c>
       <c r="T15" t="n">
+        <v>48</v>
+      </c>
+      <c r="U15" t="n">
         <v>100</v>
       </c>
-      <c r="U15" t="n">
+      <c r="V15" t="n">
         <v>1129311</v>
       </c>
-      <c r="V15" t="n">
+      <c r="W15" t="n">
         <v>70386</v>
       </c>
-      <c r="W15" t="n">
+      <c r="X15" t="n">
         <v>49235</v>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="Y15" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>
@@ -9232,18 +9271,21 @@
         <v>1.65</v>
       </c>
       <c r="T16" t="n">
+        <v>48</v>
+      </c>
+      <c r="U16" t="n">
         <v>100</v>
       </c>
-      <c r="U16" t="n">
+      <c r="V16" t="n">
         <v>484330</v>
       </c>
-      <c r="V16" t="n">
+      <c r="W16" t="n">
         <v>59039</v>
       </c>
-      <c r="W16" t="n">
+      <c r="X16" t="n">
         <v>28083</v>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="Y16" t="inlineStr">
         <is>
           <t>5/2/3</t>
         </is>

</xml_diff>